<commit_message>
Astute Tanda 1: +28 contactos clave (commodity buyers electronica) + columna Prioridad; dedup Prokure
</commit_message>
<xml_diff>
--- a/GrowProkure/04-GoToMarket/Astute_Tanda1_contactos.xlsx
+++ b/GrowProkure/04-GoToMarket/Astute_Tanda1_contactos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tanda 1 - Astute" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tanda 1 - Astute" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,36 +462,31 @@
           <t>Telefono</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kimball Electronics</t>
+          <t>KOSTAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Raul Escobedo</t>
+          <t>Gabriel Aragon Montiel</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Supervisor, Sourcing</t>
+          <t>Senior Electronics Commodity Buyer</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Reynosa</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Tamaulipas</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,44 +496,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>raul.escobedo@kimballelectronics.com</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>(956) 205-4245</t>
+          <t>g.montiel@kostal.com</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kimball Electronics</t>
+          <t>KOSTAL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Axel Jacobson</t>
+          <t>Miriam Rojas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Material Quote Specialist and NPI Leader</t>
+          <t>Strategic Electronic Purchasing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Reynosa</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Tamaulipas</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -548,44 +533,34 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>axel.jacobson@kimball.com</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>(973) 380-5588</t>
+          <t>m.rojas@kostal.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kimball Electronics</t>
+          <t>Magna</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Eduardo Solis</t>
+          <t>Ana Sanchez Mendoza</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Materials Supervisor</t>
+          <t>Global Director, Commodity, Electronics</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Reynosa</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Tamaulipas</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -595,44 +570,34 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>eduardo.solis@kimballelectronics.com</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>(760) 420-6736</t>
+          <t>ana.mendoza@magna.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Melecs</t>
+          <t>Mahle</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Elizabeth Leon</t>
+          <t>Jessica Raquel Zavala</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Operational Purchaser Coordinator</t>
+          <t>Electronic Commodity Buyer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Corregidora</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -642,44 +607,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>elizabeth.leon@melecs.com</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>+52 442 338 1552</t>
+          <t>jessica.raquel.zavala@mahle.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Melecs</t>
+          <t>MAHLE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lucia Morales</t>
+          <t>Mosiah Sosa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Operational Purchaser</t>
+          <t>Electronics/Electrical Commodity Buyer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Corregidora</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -689,44 +644,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>lucia.morales@melecs.com</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>+52 442 728 9640</t>
+          <t>mosiah.sosa@mahle.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bitron</t>
+          <t>Sumitomo Electric (SEWS)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Edith Moreno</t>
+          <t>Cecilia Ocampo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Manager, Purchasing</t>
+          <t>Components Buyer</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -736,44 +681,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>edith.moreno@bitron.com.mx</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>+52 442 227 4653</t>
+          <t>cocampo@sewsus.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bitron</t>
+          <t>Volvo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kenia Morales</t>
+          <t>Olivier Negri</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Commodity Buyer</t>
+          <t>Global Manager Purchasing Commodity, Electronics</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,39 +718,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>kenia.morales@bitron.com</t>
+          <t>olivier.negri@volvo.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bitron</t>
+          <t>Wabtec</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Celia Martinez</t>
+          <t>Gerardo Navarro</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Materials &amp; Customer Service Manager</t>
+          <t>Senior Electronics Components Commodity Leader</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -825,39 +755,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>celia.martinez@bitron.com</t>
+          <t>gerardo.navarro@wabtec.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kostal (Electro-Mobility)</t>
+          <t>Wabtec</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Omar Campos</t>
+          <t>Lezly Salas</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Director, Supply Chain</t>
+          <t>Lead Electronics Commodity Manager</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -867,44 +792,34 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>o.campos@kostal.com</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>+52 442 467 0724</t>
+          <t>lezly.salas@wabtec.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kostal (Electro-Mobility)</t>
+          <t>ZF</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Juan Luis Serrano</t>
+          <t>Carlos Tavares</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Director, Project Purchasing</t>
+          <t>Senior Global Commodity Manager Electronics</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -914,44 +829,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ju.serrano@kostal.com</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>+52 442 196 0470</t>
+          <t>carlos.tavares@zf.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kostal (Electro-Mobility)</t>
+          <t>ZKW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fernanda Tellez</t>
+          <t>Maria Tetuan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Senior Sales &amp; Materials Controller</t>
+          <t>Electronics Commodity Buyer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -961,39 +866,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>f.tellez@kostal.com</t>
+          <t>maria.tetuan@zkw.mx</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kostal (Electro-Mobility)</t>
+          <t>ZKW</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Francisco Sanchez</t>
+          <t>Paola Evangelista Cruz</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Material Requirements Planning Controller</t>
+          <t>Manager, Purchasing Commodity Electronics</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1003,44 +903,34 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>f.sanchez@kostal.com</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>(442) 211-9570</t>
+          <t>paola.evangelista@zkw.mx</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EXFO Products</t>
+          <t>Brose</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alejandro Salguero</t>
+          <t>Montserrat Mendoza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Manager, Purchasing &amp; Planning</t>
+          <t>Project Buyer - Electronics</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1050,44 +940,34 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>alejandro.salguero@exfo.com</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>+52 442 561 3033</t>
+          <t>montserrat.mendoza@brose.com</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EXFO Products</t>
+          <t>Crane Payment Innovations (CPI)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ricardo Robles</t>
+          <t>Rebeca Cortez</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Senior Buyer (OPEX/CAPEX)</t>
+          <t>Global Commodity Manager - Electronics</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>El Marques</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1097,39 +977,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>ricardo.moreno-robles@exfo.com</t>
+          <t>rebeca.cortez@cranepi.com</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1 - Clave electrónicos</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Prettl Electronics</t>
+          <t>Bitron</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gabriel Tovar</t>
+          <t>Jesus Omar Navarro Avila</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Senior Purchasing Specialist</t>
+          <t>Materials Director / Supply Chain / Procurement</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Corregidora</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1139,44 +1014,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>gtovar@pas.com</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>+52 442 192 9100 ext 224</t>
+          <t>jesus.navarro@bitron.com</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Prettl Electronics</t>
+          <t>Bombardier</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Emmanuel Covarrubias</t>
+          <t>Alfonso Reyes</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Purchasing</t>
+          <t>Supply Chain Specialist</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Corregidora</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1186,44 +1051,34 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ecovarrubias@pas.com</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>+52 412 156 3900 ext 125</t>
+          <t>alfonsoreyes@bombardier.com</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Prettl Electronics</t>
+          <t>Bombardier Querétaro</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jacqueline Estrada</t>
+          <t>Jorge Montiel Castelló</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Purchasing</t>
+          <t>Procurement Leader</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Corregidora</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Queretaro</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1233,44 +1088,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>jestrada@prettl.com.mx</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>+52 442 192 9100 ext 129</t>
+          <t>jorge.montiel@aero.bombardier.com</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Continental (Mexico - varias plantas)</t>
+          <t>Bombardier Querétaro</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Salvador Larrauri</t>
+          <t>Marcelo Oliveros de la Vega</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Manager, Corporate Purchasing</t>
+          <t>Procurement &amp; Supplier Management Leader</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>MX</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1280,44 +1125,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>salvador.2.larrauri@continental.com</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>(330) 664-7032</t>
+          <t>marcelo.oliveros@aero.bombardier.com</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Continental (Mexico - varias plantas)</t>
+          <t>EXFO</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jose Lopez Solano</t>
+          <t>Alejandro Arroyo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Execution Head of Supply Chain</t>
+          <t>Purchasing and Planning Manager</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>MX</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1327,44 +1162,34 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>jose.jesus@continental.com</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>+52 826 263 0000</t>
+          <t>alejandro.arroyo@exfo.com</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Continental (Mexico - varias plantas)</t>
+          <t>FORVIA (ex-BCS)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Amed Salas</t>
+          <t>Jocelyn Olivas Aguinaga</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Manager, Advance Supply Chain</t>
+          <t>Project Purchasing Leader</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>MX</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1374,44 +1199,34 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>amed.salas@continental-corporation.com</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>+52 631 311 9323</t>
+          <t>jocelyn.olivas@forvia.com</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Continental (Guadalajara)</t>
+          <t>Forvia Hella</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Luis Villalpando</t>
+          <t>Adriana Camarena Aguirre</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Manager, Supply Chain</t>
+          <t>Head of Purchasing</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Guadalajara</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Jalisco</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1421,44 +1236,34 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>luis.villalpando@continental-corporation.com</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>+52 33 3050 6218</t>
+          <t>adriana.aguirre@forvia.com</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Forvia Hella</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Wilfrido Serrano</t>
+          <t>Keren Cruz</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Global Manager, Procurement</t>
+          <t>Project Manager, Purchasing</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Hermosillo</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Sonora</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1468,44 +1273,34 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>wserrano@te.com</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>+52 662 319 5560</t>
+          <t>keren.sotocruz@forvia.com</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Hella</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alejandra Cheno</t>
+          <t>Eduardo Sanchez</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Manager, Commodity &amp; SSA</t>
+          <t>Supply Chain Manager</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Guaymas</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Sonora</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1515,44 +1310,34 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>alejandra.cheno@te.com</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>+52 622 225 4200 ext 4456</t>
+          <t>eduardo.sanchez@hella.com</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Hella</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jorge Mendoza Plaza</t>
+          <t>Herson Macias</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Senior Manager, Strategic Sourcing</t>
+          <t>Head of Planning Logistics</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Sonora</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Sonora</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1562,44 +1347,34 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>enrique.mendoza@te.com</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>+52 662 500 3732</t>
+          <t>macias.herson@hella.com</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Hella</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Arantxa Angulo</t>
+          <t>Jimena Tonix</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Manager, Strategic Sourcing Corporate</t>
+          <t>Head of Planning</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Sonora</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Sonora</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1609,44 +1384,34 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>arantxa.angulo@te.com</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>(662) 475-3431</t>
+          <t>jimena.tonix@hella.com</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Hella</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Marcos Quintana</t>
+          <t>Said Rivera</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Manager, Strategic Sourcing</t>
+          <t>Tooling &amp; Equipment Procurement Specialist</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Sonora</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Sonora</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1656,44 +1421,34 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>marcos.quintana@te.com</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>+52 662 500 3634</t>
+          <t>said.rivera@hella.com</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bosch (planta n/e)</t>
+          <t>Hella (Forvia Hella)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Leandro Carreira</t>
+          <t>Cain Camargo</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Head of Purchasing (North America)</t>
+          <t>Indirect Purchasing Investment Head (Americas)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>MX</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1703,39 +1458,34 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>leandro.carreira@bosch.com</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>(843) 607-4158 [NO LLAMAR movil]</t>
+          <t>cain.camargo@forvia.com</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bosch (corporativo)</t>
+          <t>Hella (Forvia Hella)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Marko Zivkovic</t>
+          <t>Carlos Vite Lara</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Senior Manager, Project Purchasing</t>
+          <t>Manager, Commodity Purchasing (Americas)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Alemania</t>
+          <t>Compras / Electrónica</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1745,29 +1495,29 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>marko.zivkovic@bosch.com</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>+49 711 81156920</t>
+          <t>carlosmanuel.lara@forvia.com</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2 - Decisor compras</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bosch (Toluca)</t>
+          <t>Kimball Electronics</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jose Del Valle Cuenca</t>
+          <t>Raul Escobedo</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Manager, Project Purchasing</t>
+          <t>Supervisor, Sourcing</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1777,12 +1527,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Toluca</t>
+          <t>Reynosa</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Estado de Mexico</t>
+          <t>Tamaulipas</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1792,44 +1542,49 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>jose.delvalle@bosch.com</t>
+          <t>raul.escobedo@kimballelectronics.com</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>+52 722 702 4196</t>
+          <t>(956) 205-4245</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sensata Technologies</t>
+          <t>Kimball Electronics</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Elizabeth Tovar</t>
+          <t>Axel Jacobson</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Senior Manager, Procurement (Ags Site)</t>
+          <t>Material Quote Specialist and NPI Leader</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
+          <t>Materiales / Planeación</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aguascalientes</t>
+          <t>Reynosa</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Aguascalientes</t>
+          <t>Tamaulipas</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1839,44 +1594,49 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>elizabethtovar@sensata.com</t>
+          <t>axel.jacobson@kimball.com</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>+52 449 910 5500 ext 5916</t>
+          <t>(973) 380-5588</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sensata Technologies</t>
+          <t>Kimball Electronics</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Carlos Robles</t>
+          <t>Eduardo Solis</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Director, Purchasing</t>
+          <t>Materials Supervisor</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
+          <t>Materiales / Planeación</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>Reynosa</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>Tamaulipas</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1886,29 +1646,34 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>c.robles@sensata.com</t>
+          <t>eduardo.solis@kimballelectronics.com</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>+52 222 152 9182</t>
+          <t>(760) 420-6736</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sensata Technologies</t>
+          <t>Melecs</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Isaac Chavez</t>
+          <t>Elizabeth Leon</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Global Manager, Commodity</t>
+          <t>Operational Purchaser Coordinator</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1918,12 +1683,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>Corregidora</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Baja California</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1933,29 +1698,34 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>isaacchavez@sensata.com</t>
+          <t>elizabeth.leon@melecs.com</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>+52 664 682 2190 ext 41422</t>
+          <t>+52 442 338 1552</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sensata Technologies</t>
+          <t>Melecs</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Wendy Aspeitia</t>
+          <t>Lucia Morales</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Global Manager, Procurement</t>
+          <t>Operational Purchaser</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1965,12 +1735,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>Corregidora</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Baja California</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1980,44 +1750,49 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>wendy.aspeitia@sensata.com</t>
+          <t>lucia.morales@melecs.com</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>+52 664 123 5946</t>
+          <t>+52 442 728 9640</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sensata Technologies</t>
+          <t>Bitron</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jose Castillo</t>
+          <t>Edith Moreno</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Director, Supply Chain</t>
+          <t>Manager, Purchasing</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
+          <t>Compras / Sourcing</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>El Marques</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2027,24 +1802,34 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>jcastillomacias@sensata.com</t>
+          <t>edith.moreno@bitron.com.mx</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>+52 442 227 4653</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marelli (Calsonic Kansei)</t>
+          <t>Bitron</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>David Aranda</t>
+          <t>Kenia Morales</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Division NAFTA Electronics Head of Purchasing</t>
+          <t>Commodity Buyer</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2054,12 +1839,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Aguascalientes</t>
+          <t>El Marques</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Aguascalientes</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2069,44 +1854,44 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>david.aranda@marelli.com</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>+52 449 500 3516</t>
+          <t>kenia.morales@bitron.com</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marelli (Calsonic Kansei)</t>
+          <t>Bitron</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Armando Lorttia</t>
+          <t>Celia Martinez</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Manager, Purchasing</t>
+          <t>Materials &amp; Customer Service Manager</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
+          <t>Materiales / Planeación</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ciudad Juarez</t>
+          <t>El Marques</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Chihuahua</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2116,44 +1901,44 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>armando.lorttia@marelli.com</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>+52 656 388 2696</t>
+          <t>celia.martinez@bitron.com</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Marelli (Calsonic Kansei)</t>
+          <t>Kostal (Electro-Mobility)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Jose Lozano</t>
+          <t>Omar Campos</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Manager, Purchasing</t>
+          <t>Director, Supply Chain</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
+          <t>Materiales / Planeación</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Saltillo</t>
+          <t>El Marques</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Coahuila</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2163,44 +1948,49 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>jose.lozano@marelli.com</t>
+          <t>o.campos@kostal.com</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>+52 844 444 6733</t>
+          <t>+52 442 467 0724</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Marelli (Calsonic Kansei)</t>
+          <t>Kostal (Electro-Mobility)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Aldo Martinez Ochoa</t>
+          <t>Juan Luis Serrano</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Head of Materials</t>
+          <t>Director, Project Purchasing</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Materiales / Planeación</t>
+          <t>Compras / Sourcing</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>El Marques</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2210,54 +2000,1500 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>aldo.martinez@marelli.com</t>
+          <t>ju.serrano@kostal.com</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>+52 222 304 9631</t>
+          <t>+52 442 196 0470</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>Kostal (Electro-Mobility)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Fernanda Tellez</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Senior Sales &amp; Materials Controller</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>El Marques</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>f.tellez@kostal.com</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Kostal (Electro-Mobility)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Francisco Sanchez</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Material Requirements Planning Controller</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>El Marques</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>f.sanchez@kostal.com</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>(442) 211-9570</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>EXFO Products</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Alejandro Salguero</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Manager, Purchasing &amp; Planning</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>El Marques</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>alejandro.salguero@exfo.com</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>+52 442 561 3033</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>EXFO Products</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Ricardo Robles</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Senior Buyer (OPEX/CAPEX)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>El Marques</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>ricardo.moreno-robles@exfo.com</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Prettl Electronics</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Gabriel Tovar</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Senior Purchasing Specialist</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Corregidora</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>gtovar@pas.com</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>+52 442 192 9100 ext 224</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Prettl Electronics</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Emmanuel Covarrubias</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Corregidora</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>ecovarrubias@pas.com</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>+52 412 156 3900 ext 125</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Prettl Electronics</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Jacqueline Estrada</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Corregidora</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Queretaro</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>jestrada@prettl.com.mx</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>+52 442 192 9100 ext 129</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Continental (Mexico - varias plantas)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Salvador Larrauri</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Manager, Corporate Purchasing</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>salvador.2.larrauri@continental.com</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>(330) 664-7032</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Continental (Mexico - varias plantas)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Jose Lopez Solano</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Execution Head of Supply Chain</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>jose.jesus@continental.com</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>+52 826 263 0000</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Continental (Mexico - varias plantas)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Amed Salas</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Manager, Advance Supply Chain</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>amed.salas@continental-corporation.com</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>+52 631 311 9323</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Continental (Guadalajara)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Luis Villalpando</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Manager, Supply Chain</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Jalisco</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>luis.villalpando@continental-corporation.com</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>+52 33 3050 6218</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Wilfrido Serrano</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Global Manager, Procurement</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Hermosillo</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>wserrano@te.com</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>+52 662 319 5560</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Alejandra Cheno</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Manager, Commodity &amp; SSA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Guaymas</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>alejandra.cheno@te.com</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>+52 622 225 4200 ext 4456</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Jorge Mendoza Plaza</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Senior Manager, Strategic Sourcing</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>enrique.mendoza@te.com</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>+52 662 500 3732</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Arantxa Angulo</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Manager, Strategic Sourcing Corporate</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>arantxa.angulo@te.com</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>(662) 475-3431</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Marcos Quintana</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Manager, Strategic Sourcing</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Sonora</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>marcos.quintana@te.com</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>+52 662 500 3634</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Bosch (planta n/e)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Leandro Carreira</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Head of Purchasing (North America)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>leandro.carreira@bosch.com</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>(843) 607-4158 [NO LLAMAR movil]</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Bosch (corporativo)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Marko Zivkovic</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Senior Manager, Project Purchasing</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>marko.zivkovic@bosch.com</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>+49 711 81156920</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Bosch (Toluca)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Jose Del Valle Cuenca</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Manager, Project Purchasing</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Estado de Mexico</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>jose.delvalle@bosch.com</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>+52 722 702 4196</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Sensata Technologies</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Elizabeth Tovar</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Senior Manager, Procurement (Ags Site)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Aguascalientes</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Aguascalientes</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>elizabethtovar@sensata.com</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>+52 449 910 5500 ext 5916</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Sensata Technologies</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Carlos Robles</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Director, Purchasing</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>c.robles@sensata.com</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>+52 222 152 9182</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Sensata Technologies</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Isaac Chavez</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Global Manager, Commodity</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Baja California</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>isaacchavez@sensata.com</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>+52 664 682 2190 ext 41422</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Sensata Technologies</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Wendy Aspeitia</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Global Manager, Procurement</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Baja California</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>wendy.aspeitia@sensata.com</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>+52 664 123 5946</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Sensata Technologies</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Jose Castillo</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Director, Supply Chain</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>jcastillomacias@sensata.com</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>Marelli (Calsonic Kansei)</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>David Aranda</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Division NAFTA Electronics Head of Purchasing</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Aguascalientes</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Aguascalientes</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>david.aranda@marelli.com</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>+52 449 500 3516</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Marelli (Calsonic Kansei)</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Armando Lorttia</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Manager, Purchasing</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Ciudad Juarez</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Chihuahua</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>armando.lorttia@marelli.com</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>+52 656 388 2696</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Marelli (Calsonic Kansei)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Jose Lozano</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Manager, Purchasing</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Compras / Sourcing</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Saltillo</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Coahuila</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>jose.lozano@marelli.com</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>+52 844 444 6733</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Marelli (Calsonic Kansei)</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Aldo Martinez Ochoa</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Head of Materials</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Materiales / Planeación</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>aldo.martinez@marelli.com</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>+52 222 304 9631</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Marelli (Calsonic Kansei)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>Lucia Zayarzabal</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>Senior Manager, Regional Supply Chain</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>Materiales / Planeación</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
         <is>
           <t>lucia.zayarzabal@marelli.com</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>3 - Estudio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Astute Tanda 1: quitar TE Connectivity y Sensata (feedback Carlos)
</commit_message>
<xml_diff>
--- a/GrowProkure/04-GoToMarket/Astute_Tanda1_contactos.xlsx
+++ b/GrowProkure/04-GoToMarket/Astute_Tanda1_contactos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2579,17 +2579,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Bosch (planta n/e)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Wilfrido Serrano</t>
+          <t>Leandro Carreira</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Global Manager, Procurement</t>
+          <t>Head of Purchasing (North America)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2599,12 +2599,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hermosillo</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>wserrano@te.com</t>
+          <t>leandro.carreira@bosch.com</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>+52 662 319 5560</t>
+          <t>(843) 607-4158 [NO LLAMAR movil]</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2631,17 +2631,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Bosch (corporativo)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alejandra Cheno</t>
+          <t>Marko Zivkovic</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Manager, Commodity &amp; SSA</t>
+          <t>Senior Manager, Project Purchasing</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2651,12 +2651,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Guaymas</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Sonora</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2666,12 +2661,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>alejandra.cheno@te.com</t>
+          <t>marko.zivkovic@bosch.com</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>+52 622 225 4200 ext 4456</t>
+          <t>+49 711 81156920</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2683,17 +2678,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Bosch (Toluca)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jorge Mendoza Plaza</t>
+          <t>Jose Del Valle Cuenca</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Senior Manager, Strategic Sourcing</t>
+          <t>Manager, Project Purchasing</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2703,12 +2698,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>Toluca</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>Estado de Mexico</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2718,12 +2713,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>enrique.mendoza@te.com</t>
+          <t>jose.delvalle@bosch.com</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>+52 662 500 3732</t>
+          <t>+52 722 702 4196</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2735,17 +2730,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Marelli (Calsonic Kansei)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Arantxa Angulo</t>
+          <t>David Aranda</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Manager, Strategic Sourcing Corporate</t>
+          <t>Division NAFTA Electronics Head of Purchasing</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2755,12 +2750,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>Aguascalientes</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>Aguascalientes</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2770,12 +2765,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>arantxa.angulo@te.com</t>
+          <t>david.aranda@marelli.com</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>(662) 475-3431</t>
+          <t>+52 449 500 3516</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2787,17 +2782,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>Marelli (Calsonic Kansei)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Marcos Quintana</t>
+          <t>Armando Lorttia</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Manager, Strategic Sourcing</t>
+          <t>Manager, Purchasing</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2807,12 +2802,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>Ciudad Juarez</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sonora</t>
+          <t>Chihuahua</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2822,12 +2817,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>marcos.quintana@te.com</t>
+          <t>armando.lorttia@marelli.com</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>+52 662 500 3634</t>
+          <t>+52 656 388 2696</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2839,17 +2834,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Bosch (planta n/e)</t>
+          <t>Marelli (Calsonic Kansei)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Leandro Carreira</t>
+          <t>Jose Lozano</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Head of Purchasing (North America)</t>
+          <t>Manager, Purchasing</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2859,12 +2854,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>Saltillo</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>Coahuila</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2874,12 +2869,12 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>leandro.carreira@bosch.com</t>
+          <t>jose.lozano@marelli.com</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>(843) 607-4158 [NO LLAMAR movil]</t>
+          <t>+52 844 444 6733</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -2891,27 +2886,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bosch (corporativo)</t>
+          <t>Marelli (Calsonic Kansei)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Marko Zivkovic</t>
+          <t>Aldo Martinez Ochoa</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Senior Manager, Project Purchasing</t>
+          <t>Head of Materials</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
+          <t>Materiales / Planeación</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>MX</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2921,12 +2921,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>marko.zivkovic@bosch.com</t>
+          <t>aldo.martinez@marelli.com</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>+49 711 81156920</t>
+          <t>+52 222 304 9631</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -2938,32 +2938,32 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bosch (Toluca)</t>
+          <t>Marelli (Calsonic Kansei)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Jose Del Valle Cuenca</t>
+          <t>Lucia Zayarzabal</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Manager, Project Purchasing</t>
+          <t>Senior Manager, Regional Supply Chain</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Compras / Sourcing</t>
+          <t>Materiales / Planeación</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Toluca</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Estado de Mexico</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2973,525 +2973,10 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>jose.delvalle@bosch.com</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>+52 722 702 4196</t>
+          <t>lucia.zayarzabal@marelli.com</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Sensata Technologies</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Elizabeth Tovar</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Senior Manager, Procurement (Ags Site)</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Aguascalientes</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Aguascalientes</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>elizabethtovar@sensata.com</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>+52 449 910 5500 ext 5916</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Sensata Technologies</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Carlos Robles</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Director, Purchasing</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>c.robles@sensata.com</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>+52 222 152 9182</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Sensata Technologies</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Isaac Chavez</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Global Manager, Commodity</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Baja California</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>isaacchavez@sensata.com</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>+52 664 682 2190 ext 41422</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Sensata Technologies</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Wendy Aspeitia</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Global Manager, Procurement</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Baja California</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>wendy.aspeitia@sensata.com</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>+52 664 123 5946</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Sensata Technologies</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Jose Castillo</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Director, Supply Chain</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>jcastillomacias@sensata.com</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Marelli (Calsonic Kansei)</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>David Aranda</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Division NAFTA Electronics Head of Purchasing</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Aguascalientes</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Aguascalientes</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>david.aranda@marelli.com</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>+52 449 500 3516</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Marelli (Calsonic Kansei)</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Armando Lorttia</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Manager, Purchasing</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Ciudad Juarez</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Chihuahua</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>armando.lorttia@marelli.com</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>+52 656 388 2696</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Marelli (Calsonic Kansei)</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Jose Lozano</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Manager, Purchasing</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Compras / Sourcing</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Saltillo</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Coahuila</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>jose.lozano@marelli.com</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>+52 844 444 6733</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Marelli (Calsonic Kansei)</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Aldo Martinez Ochoa</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Head of Materials</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>aldo.martinez@marelli.com</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>+52 222 304 9631</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>3 - Estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Marelli (Calsonic Kansei)</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Lucia Zayarzabal</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Senior Manager, Regional Supply Chain</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Materiales / Planeación</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>lucia.zayarzabal@marelli.com</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
         <is>
           <t>3 - Estudio</t>
         </is>

</xml_diff>